<commit_message>
Track decision timestamps and chart hourly queue size
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kyc-review-app/data/KYC_review.xlsx
+++ b/kyc-review-app/data/KYC_review.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:J101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,9 @@
       <c r="I1" t="str">
         <v>Entered Queue</v>
       </c>
+      <c r="J1" t="str">
+        <v>Decided At</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -543,6 +546,9 @@
       <c r="I5" s="1">
         <v>46266.68251157407</v>
       </c>
+      <c r="J5" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1186,6 +1192,9 @@
       <c r="I28" s="1">
         <v>46266.71332175926</v>
       </c>
+      <c r="J28" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -1244,6 +1253,9 @@
       <c r="I30" s="1">
         <v>46266.7855787037</v>
       </c>
+      <c r="J30" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -1328,6 +1340,9 @@
       <c r="I33" s="1">
         <v>46266.78171296296</v>
       </c>
+      <c r="J33" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -1858,6 +1873,9 @@
       <c r="I52" s="1">
         <v>46266.70075231481</v>
       </c>
+      <c r="J52" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -2084,6 +2102,9 @@
       <c r="I60" s="1">
         <v>46266.73094907407</v>
       </c>
+      <c r="J60" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -3176,6 +3197,9 @@
       <c r="I99" s="1">
         <v>46266.76832175926</v>
       </c>
+      <c r="J99" s="1" t="d">
+        <v>2026-09-03T12:22:00.214Z</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100">
@@ -3235,7 +3259,7 @@
   </sheetData>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track decision timestamps and chart queue size by hour
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kyc-review-app/data/KYC_review.xlsx
+++ b/kyc-review-app/data/KYC_review.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:J101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,9 @@
       <c r="I1" t="str">
         <v>Entered Queue</v>
       </c>
+      <c r="J1" t="str">
+        <v>Decided At</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -543,6 +546,9 @@
       <c r="I5" s="1">
         <v>46266.68251157407</v>
       </c>
+      <c r="J5" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1186,6 +1192,9 @@
       <c r="I28" s="1">
         <v>46266.71332175926</v>
       </c>
+      <c r="J28" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -1244,6 +1253,9 @@
       <c r="I30" s="1">
         <v>46266.7855787037</v>
       </c>
+      <c r="J30" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -1328,6 +1340,9 @@
       <c r="I33" s="1">
         <v>46266.78171296296</v>
       </c>
+      <c r="J33" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -1858,6 +1873,9 @@
       <c r="I52" s="1">
         <v>46266.70075231481</v>
       </c>
+      <c r="J52" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -2084,6 +2102,9 @@
       <c r="I60" s="1">
         <v>46266.73094907407</v>
       </c>
+      <c r="J60" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -3176,6 +3197,9 @@
       <c r="I99" s="1">
         <v>46266.76832175926</v>
       </c>
+      <c r="J99" s="1">
+        <v>46268.59886574074</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100">
@@ -3235,7 +3259,7 @@
   </sheetData>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>